<commit_message>
docs: update reve unit economics assumptions
</commit_message>
<xml_diff>
--- a/docs/business/unit-economics-june-model.xlsx
+++ b/docs/business/unit-economics-june-model.xlsx
@@ -73,8 +73,8 @@
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="37" customWidth="1"/>
-    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="4" max="4" width="35" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -110,7 +110,9 @@
           <t>usd_rub</t>
         </is>
       </c>
-      <c r="B2"/>
+      <c r="B2" s="2">
+        <v>100</v>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>RUB/USD</t>
@@ -118,12 +120,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Курс для planning</t>
+          <t>Conservative planning</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Заполняется вручную</t>
+          <t>Округлено вверх</t>
         </is>
       </c>
     </row>
@@ -209,7 +211,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -218,12 +220,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Planning hypothesis</t>
+          <t>Current backend check</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Доля Remix Fast в B2C</t>
+          <t>Сейчас fast не используется</t>
         </is>
       </c>
     </row>
@@ -234,7 +236,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -243,12 +245,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Planning hypothesis</t>
+          <t>Current backend check</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Доля Remix в B2C</t>
+          <t>Текущий backend: /v1/image/remix, 30 credits</t>
         </is>
       </c>
     </row>
@@ -283,7 +285,9 @@
           <t>fallback_attempt_usd</t>
         </is>
       </c>
-      <c r="B9"/>
+      <c r="B9" s="2">
+        <v>0.2</v>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>USD</t>
@@ -291,12 +295,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Provider docs/billing</t>
+          <t>Rounded placeholder</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OpenAI или другой fallback</t>
+          <t>OpenAI/high-quality fallback placeholder</t>
         </is>
       </c>
     </row>
@@ -356,7 +360,9 @@
           <t>attempts_per_success</t>
         </is>
       </c>
-      <c r="B12"/>
+      <c r="B12" s="2">
+        <v>2</v>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>x</t>
@@ -364,12 +370,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>30-50 test pairs / production usage</t>
+          <t>Rounded up estimate</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Среднее число попыток на successful render</t>
+          <t>До теста 30-50 пар</t>
         </is>
       </c>
     </row>
@@ -379,7 +385,9 @@
           <t>technical_failure_rate</t>
         </is>
       </c>
-      <c r="B13"/>
+      <c r="B13" s="2">
+        <v>0.15</v>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>%</t>
@@ -387,7 +395,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>failed / total_jobs</t>
+          <t>Rounded up estimate</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -402,7 +410,9 @@
           <t>payment_fee_rate</t>
         </is>
       </c>
-      <c r="B14"/>
+      <c r="B14" s="2">
+        <v>0.05</v>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>%</t>
@@ -410,7 +420,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Robokassa contract/dashboard</t>
+          <t>Rounded up until Robokassa tariff</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -425,7 +435,9 @@
           <t>payment_fee_fixed</t>
         </is>
       </c>
-      <c r="B15"/>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>RUB</t>
@@ -448,7 +460,9 @@
           <t>infra_monthly</t>
         </is>
       </c>
-      <c r="B16"/>
+      <c r="B16" s="2">
+        <v>3000</v>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>RUB/month</t>
@@ -456,12 +470,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>Rounded reserve</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>Render/Supabase/Redis/Storage</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Месячная инфраструктура</t>
         </is>
       </c>
     </row>
@@ -471,7 +485,9 @@
           <t>paid_renders_month</t>
         </is>
       </c>
-      <c r="B17"/>
+      <c r="B17" s="2">
+        <v>1000</v>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>renders</t>
@@ -479,7 +495,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sales plan / actual usage</t>
+          <t>Launch planning base</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -494,7 +510,9 @@
           <t>support_buffer_render</t>
         </is>
       </c>
-      <c r="B18"/>
+      <c r="B18" s="2">
+        <v>5</v>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>RUB</t>
@@ -502,7 +520,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Support estimate</t>
+          <t>Rounded reserve</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -517,7 +535,9 @@
           <t>free_trial_renders</t>
         </is>
       </c>
-      <c r="B19"/>
+      <c r="B19" s="2">
+        <v>100</v>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>renders</t>
@@ -540,7 +560,9 @@
           <t>refund_rate</t>
         </is>
       </c>
-      <c r="B20"/>
+      <c r="B20" s="2">
+        <v>0.05</v>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>%</t>
@@ -548,7 +570,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Payment/refund events</t>
+          <t>Rounded up estimate</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -563,7 +585,9 @@
           <t>target_margin_founder</t>
         </is>
       </c>
-      <c r="B21"/>
+      <c r="B21" s="2">
+        <v>150</v>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>RUB</t>
@@ -586,7 +610,9 @@
           <t>internal_credit_cost_rub</t>
         </is>
       </c>
-      <c r="B22"/>
+      <c r="B22" s="2">
+        <v>25</v>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>RUB</t>
@@ -615,7 +641,7 @@
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="5" max="5" width="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -683,7 +709,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>cheap B2C baseline</t>
+          <t>future cheap baseline, not current backend</t>
         </is>
       </c>
     </row>
@@ -704,7 +730,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>quality B2C baseline</t>
+          <t>current B2C backend baseline</t>
         </is>
       </c>
     </row>
@@ -759,7 +785,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="2" max="2" width="47" customWidth="1"/>
     <col min="3" max="3" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -997,8 +1023,12 @@
           <t>First paid step</t>
         </is>
       </c>
-      <c r="C3"/>
-      <c r="D3"/>
+      <c r="C3" s="2">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2">
+        <v>3</v>
+      </c>
       <c r="E3" s="2">
         <f>C3*Inputs!B14+Inputs!B15</f>
       </c>
@@ -1063,8 +1093,12 @@
           <t>Active shoppers</t>
         </is>
       </c>
-      <c r="C5"/>
-      <c r="D5"/>
+      <c r="C5" s="2">
+        <v>499</v>
+      </c>
+      <c r="D5" s="2">
+        <v>20</v>
+      </c>
       <c r="E5" s="2">
         <f>C5*Inputs!B14+Inputs!B15</f>
       </c>
@@ -1094,8 +1128,12 @@
           <t>Later</t>
         </is>
       </c>
-      <c r="C6"/>
-      <c r="D6"/>
+      <c r="C6" s="2">
+        <v>990</v>
+      </c>
+      <c r="D6" s="2">
+        <v>50</v>
+      </c>
       <c r="E6" s="2">
         <f>C6*Inputs!B14+Inputs!B15</f>
       </c>
@@ -1123,10 +1161,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="46" customWidth="1"/>
+    <col min="5" max="5" width="47" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="32" customWidth="1"/>
   </cols>
@@ -1193,7 +1231,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>fast catalog preview</t>
+          <t>future fast catalog preview</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1260,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>default B2B2C quality</t>
+          <t>current/default quality</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1366,7 @@
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="46" customWidth="1"/>
+    <col min="8" max="8" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1407,7 +1445,7 @@
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1487,7 +1525,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Current: 100% reve_remix</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1552,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Estimate: 2.0</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1579,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Estimate: 15%</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1606,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD from DB</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1633,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Estimate: 5%</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1754,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>